<commit_message>
extra controle op kinderen
</commit_message>
<xml_diff>
--- a/roulette2025.xlsx
+++ b/roulette2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tacobakker/PycharmProjects/Kitchenroulette/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E59A597E-610C-0D45-954C-F56058224C06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6006A83-4001-F644-A29B-7F161948BD9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="6760" yWindow="3720" windowWidth="27440" windowHeight="16240" xr2:uid="{00D46D12-6840-BD4A-9AFF-D7800ADFA46E}"/>
   </bookViews>
@@ -198,7 +198,7 @@
     <t>kids</t>
   </si>
   <si>
-    <t>kidsmee</t>
+    <t>kids_mee</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Laatste wijzigingen voor voorjaarsronde
</commit_message>
<xml_diff>
--- a/roulette2025.xlsx
+++ b/roulette2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11207"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10308"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tacobakker/PycharmProjects/Kitchenroulette/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F6006A83-4001-F644-A29B-7F161948BD9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF1D2274-7E2B-9940-BAB3-61FDDE83783E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6760" yWindow="3720" windowWidth="27440" windowHeight="16240" xr2:uid="{00D46D12-6840-BD4A-9AFF-D7800ADFA46E}"/>
+    <workbookView xWindow="0" yWindow="680" windowWidth="34200" windowHeight="19720" xr2:uid="{00D46D12-6840-BD4A-9AFF-D7800ADFA46E}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="234" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="210" uniqueCount="76">
   <si>
     <t>naam</t>
   </si>
@@ -199,6 +199,72 @@
   </si>
   <si>
     <t>kids_mee</t>
+  </si>
+  <si>
+    <t>Jennifer, Tineke en Kees</t>
+  </si>
+  <si>
+    <t>Frank en Violette</t>
+  </si>
+  <si>
+    <t>Warder 134</t>
+  </si>
+  <si>
+    <t>Harry en Anja</t>
+  </si>
+  <si>
+    <t>Warder 187</t>
+  </si>
+  <si>
+    <t>Tim en Lotte</t>
+  </si>
+  <si>
+    <t>Pieter en Clara + 2 kids</t>
+  </si>
+  <si>
+    <t>Warder 9</t>
+  </si>
+  <si>
+    <t>Tim en Angelique</t>
+  </si>
+  <si>
+    <t>Ernst en Susanna</t>
+  </si>
+  <si>
+    <t>IJsselmeerdijk 8</t>
+  </si>
+  <si>
+    <t>Warder 18</t>
+  </si>
+  <si>
+    <t>Hans en Marjan</t>
+  </si>
+  <si>
+    <t>Rosa + 2 kids</t>
+  </si>
+  <si>
+    <t>Geen koriander, komkommer, tropische vruchten, spruitjes en witlof</t>
+  </si>
+  <si>
+    <t>Geen garnalen, zeevruchten, wild</t>
+  </si>
+  <si>
+    <t>Geen scherp eten en geen bereide paprika (gekookt of gebakken)</t>
+  </si>
+  <si>
+    <t>1 volwassene en 2 kids</t>
+  </si>
+  <si>
+    <t>Nemen een klein hondje mee. Geen vis, schaal en schelpdieren</t>
+  </si>
+  <si>
+    <t>Hebben 2 kinderen</t>
+  </si>
+  <si>
+    <t>Warder 82</t>
+  </si>
+  <si>
+    <t>Geen koriander</t>
   </si>
 </sst>
 </file>
@@ -594,11 +660,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07DA02DF-3BCB-1F40-ADDD-1E1F5BA5C8E3}">
-  <dimension ref="A1:J17"/>
+  <dimension ref="A1:J35"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="15.83203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="16" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.1640625" bestFit="1" customWidth="1"/>
@@ -639,516 +705,672 @@
       </c>
     </row>
     <row r="2" spans="1:10">
-      <c r="A2" s="4" t="s">
-        <v>5</v>
+      <c r="A2" s="2" t="s">
+        <v>64</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="2">
+        <v>2</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I2" s="2">
+        <v>4</v>
+      </c>
+      <c r="J2" s="2" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C3" s="2">
+        <v>2</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I3" s="2">
+        <v>8</v>
+      </c>
+      <c r="J3" s="2" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="2">
+        <v>2</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" s="2">
         <v>6</v>
       </c>
-      <c r="C2" s="3">
-        <v>2</v>
-      </c>
-      <c r="D2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I2" s="3">
-        <v>8</v>
-      </c>
-      <c r="J2" s="2" t="s">
+      <c r="J4" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="2">
+        <v>2</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I5" s="2">
+        <v>6</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="C6" s="2">
+        <v>3</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I6" s="2">
+        <v>8</v>
+      </c>
+      <c r="J6" s="2" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C7" s="2">
+        <v>2</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H7" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I7" s="2">
+        <v>6</v>
+      </c>
+      <c r="J7" s="2" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:10">
-      <c r="A3" s="4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B3" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="3">
-        <v>2</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I3" s="3">
-        <v>8</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="4" spans="1:10">
-      <c r="A4" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" s="3">
+    <row r="8" spans="1:10">
+      <c r="A8" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="2">
+        <v>2</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H8" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I8" s="2">
+        <v>8</v>
+      </c>
+      <c r="J8" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="2">
+        <v>2</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H9" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I9" s="2">
+        <v>6</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C10" s="2">
+        <v>2</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I10" s="2">
+        <v>6</v>
+      </c>
+      <c r="J10" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C11" s="2">
+        <v>3</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I11" s="2">
+        <v>8</v>
+      </c>
+      <c r="J11" s="2" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="2">
         <v>4</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" s="3">
-        <v>8</v>
-      </c>
-      <c r="J4" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:10">
-      <c r="A5" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="C5" s="3">
-        <v>2</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I5" s="3">
-        <v>8</v>
-      </c>
-      <c r="J5" s="2" t="s">
+      <c r="D12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H12" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="I12" s="2">
+        <v>8</v>
+      </c>
+      <c r="J12" s="2" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C13" s="2">
+        <v>2</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="H13" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I13" s="2">
+        <v>6</v>
+      </c>
+      <c r="J13" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="2">
+        <v>2</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="G14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="I14" s="2">
+        <v>6</v>
+      </c>
+      <c r="J14" s="2" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:10">
-      <c r="A6" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="C6" s="3">
-        <v>4</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H6" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I6" s="3">
-        <v>8</v>
-      </c>
-      <c r="J6" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="7" spans="1:10">
-      <c r="A7" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C7" s="3">
-        <v>2</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F7" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I7" s="3">
-        <v>8</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10">
-      <c r="A8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B8" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="C8" s="3">
-        <v>2</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H8" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I8" s="3">
-        <v>8</v>
-      </c>
-      <c r="J8" s="2" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10">
-      <c r="A9" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="C9" s="3">
-        <v>2</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F9" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H9" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I9" s="3">
-        <v>8</v>
-      </c>
-      <c r="J9" s="2" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10">
-      <c r="A10" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" s="3">
-        <v>2</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H10" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I10" s="3">
-        <v>8</v>
-      </c>
-      <c r="J10" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10">
-      <c r="A11" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C11" s="3">
-        <v>2</v>
-      </c>
-      <c r="D11" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E11" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G11" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H11" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I11" s="3">
-        <v>8</v>
-      </c>
-      <c r="J11" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10">
-      <c r="A12" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C12" s="3">
-        <v>2</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I12" s="3">
-        <v>8</v>
-      </c>
-      <c r="J12" s="2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
-      <c r="A13" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C13" s="3">
-        <v>4</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="F13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H13" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="I13" s="3">
-        <v>8</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="14" spans="1:10">
-      <c r="A14" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>41</v>
-      </c>
-      <c r="C14" s="3">
-        <v>2</v>
-      </c>
-      <c r="D14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H14" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I14" s="3">
-        <v>8</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>9</v>
-      </c>
-    </row>
     <row r="15" spans="1:10">
-      <c r="A15" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="B15" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="C15" s="3">
-        <v>2</v>
-      </c>
-      <c r="D15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="E15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="H15" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I15" s="3">
-        <v>6</v>
-      </c>
-      <c r="J15" s="2" t="s">
-        <v>18</v>
-      </c>
+      <c r="A15" s="2"/>
+      <c r="B15" s="2"/>
+      <c r="C15" s="2"/>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
     </row>
     <row r="16" spans="1:10">
-      <c r="A16" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" s="3">
-        <v>2</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E16" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F16" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G16" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H16" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I16" s="3">
-        <v>6</v>
-      </c>
-      <c r="J16" s="2" t="s">
-        <v>18</v>
-      </c>
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
     </row>
     <row r="17" spans="1:10">
-      <c r="A17" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="B17" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="C17" s="3">
-        <v>2</v>
-      </c>
-      <c r="D17" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="E17" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="F17" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="G17" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H17" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="I17" s="3">
-        <v>6</v>
-      </c>
-      <c r="J17" s="2" t="s">
-        <v>48</v>
-      </c>
+      <c r="A17" s="2"/>
+      <c r="B17" s="2"/>
+      <c r="C17" s="2"/>
+      <c r="D17" s="2"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+    </row>
+    <row r="18" spans="1:10">
+      <c r="A18" s="4"/>
+      <c r="B18" s="2"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
+      <c r="J18" s="2"/>
+    </row>
+    <row r="19" spans="1:10">
+      <c r="A19" s="4"/>
+      <c r="B19" s="2"/>
+      <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
+      <c r="J19" s="2"/>
+    </row>
+    <row r="20" spans="1:10">
+      <c r="A20" s="4"/>
+      <c r="B20" s="2"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
+      <c r="J20" s="2"/>
+    </row>
+    <row r="21" spans="1:10">
+      <c r="A21" s="4"/>
+      <c r="B21" s="2"/>
+      <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
+      <c r="J21" s="2"/>
+    </row>
+    <row r="22" spans="1:10">
+      <c r="A22" s="4"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
+      <c r="J22" s="2"/>
+    </row>
+    <row r="23" spans="1:10">
+      <c r="A23" s="4"/>
+      <c r="B23" s="2"/>
+      <c r="C23" s="3"/>
+      <c r="D23" s="3"/>
+      <c r="E23" s="3"/>
+      <c r="F23" s="3"/>
+      <c r="G23" s="3"/>
+      <c r="H23" s="3"/>
+      <c r="I23" s="3"/>
+      <c r="J23" s="2"/>
+    </row>
+    <row r="24" spans="1:10">
+      <c r="A24" s="4"/>
+      <c r="B24" s="2"/>
+      <c r="C24" s="3"/>
+      <c r="D24" s="3"/>
+      <c r="E24" s="3"/>
+      <c r="F24" s="3"/>
+      <c r="G24" s="3"/>
+      <c r="H24" s="3"/>
+      <c r="I24" s="3"/>
+      <c r="J24" s="2"/>
+    </row>
+    <row r="25" spans="1:10">
+      <c r="A25" s="4"/>
+      <c r="B25" s="2"/>
+      <c r="C25" s="3"/>
+      <c r="D25" s="3"/>
+      <c r="E25" s="3"/>
+      <c r="F25" s="3"/>
+      <c r="G25" s="3"/>
+      <c r="H25" s="3"/>
+      <c r="I25" s="3"/>
+      <c r="J25" s="2"/>
+    </row>
+    <row r="26" spans="1:10">
+      <c r="A26" s="4"/>
+      <c r="B26" s="2"/>
+      <c r="C26" s="3"/>
+      <c r="D26" s="3"/>
+      <c r="E26" s="3"/>
+      <c r="F26" s="3"/>
+      <c r="G26" s="3"/>
+      <c r="H26" s="3"/>
+      <c r="I26" s="3"/>
+      <c r="J26" s="2"/>
+    </row>
+    <row r="27" spans="1:10">
+      <c r="A27" s="4"/>
+      <c r="B27" s="2"/>
+      <c r="C27" s="3"/>
+      <c r="D27" s="3"/>
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+      <c r="G27" s="3"/>
+      <c r="H27" s="3"/>
+      <c r="I27" s="3"/>
+      <c r="J27" s="2"/>
+    </row>
+    <row r="28" spans="1:10">
+      <c r="A28" s="4"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
+      <c r="E28" s="3"/>
+      <c r="F28" s="3"/>
+      <c r="G28" s="3"/>
+      <c r="H28" s="3"/>
+      <c r="I28" s="3"/>
+      <c r="J28" s="2"/>
+    </row>
+    <row r="29" spans="1:10">
+      <c r="A29" s="4"/>
+      <c r="B29" s="2"/>
+      <c r="C29" s="3"/>
+      <c r="D29" s="3"/>
+      <c r="E29" s="3"/>
+      <c r="F29" s="3"/>
+      <c r="G29" s="3"/>
+      <c r="H29" s="3"/>
+      <c r="I29" s="3"/>
+      <c r="J29" s="2"/>
+    </row>
+    <row r="30" spans="1:10">
+      <c r="A30" s="4"/>
+      <c r="B30" s="2"/>
+      <c r="C30" s="3"/>
+      <c r="D30" s="3"/>
+      <c r="E30" s="3"/>
+      <c r="F30" s="3"/>
+      <c r="G30" s="3"/>
+      <c r="H30" s="3"/>
+      <c r="I30" s="3"/>
+      <c r="J30" s="2"/>
+    </row>
+    <row r="31" spans="1:10">
+      <c r="A31" s="4"/>
+      <c r="B31" s="2"/>
+      <c r="C31" s="3"/>
+      <c r="D31" s="3"/>
+      <c r="E31" s="3"/>
+      <c r="F31" s="3"/>
+      <c r="G31" s="3"/>
+      <c r="H31" s="3"/>
+      <c r="I31" s="3"/>
+      <c r="J31" s="2"/>
+    </row>
+    <row r="32" spans="1:10">
+      <c r="A32" s="4"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+      <c r="G32" s="3"/>
+      <c r="H32" s="3"/>
+      <c r="I32" s="3"/>
+      <c r="J32" s="2"/>
+    </row>
+    <row r="33" spans="1:10">
+      <c r="A33" s="4"/>
+      <c r="B33" s="2"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
+      <c r="I33" s="3"/>
+      <c r="J33" s="2"/>
+    </row>
+    <row r="34" spans="1:10">
+      <c r="A34" s="4"/>
+      <c r="B34" s="2"/>
+      <c r="C34" s="3"/>
+      <c r="D34" s="3"/>
+      <c r="E34" s="3"/>
+      <c r="F34" s="3"/>
+      <c r="G34" s="3"/>
+      <c r="H34" s="3"/>
+      <c r="I34" s="3"/>
+      <c r="J34" s="2"/>
+    </row>
+    <row r="35" spans="1:10">
+      <c r="A35" s="4"/>
+      <c r="B35" s="2"/>
+      <c r="C35" s="3"/>
+      <c r="D35" s="3"/>
+      <c r="E35" s="3"/>
+      <c r="F35" s="3"/>
+      <c r="G35" s="3"/>
+      <c r="H35" s="3"/>
+      <c r="I35" s="3"/>
+      <c r="J35" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>